<commit_message>
feat: show total number of questions
</commit_message>
<xml_diff>
--- a/data/questions.xlsx
+++ b/data/questions.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Vinh\Tài liệu\M500\Huấn luyện\Kiểm tra\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Tech\Projects\quiz-app\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDBD3D73-D541-461E-AF86-79B79DD0B3FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20250" windowHeight="7515" firstSheet="1" activeTab="1"/>
+    <workbookView xWindow="-28920" yWindow="840" windowWidth="29040" windowHeight="16440" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="foxz" sheetId="2" state="veryHidden" r:id="rId1"/>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="92">
   <si>
     <t>Hành trình piston ở trên tay biên chính là:</t>
   </si>
@@ -78,51 +79,15 @@
     <t>Thứ tự block xilanh và block nhiên liệu từ 1 đến 7 được sắp xếp theo thứ tự:</t>
   </si>
   <si>
-    <t>• Ý 1 và 3</t>
-  </si>
-  <si>
     <t>Tay biên chính động cơ M500 được bố trí block số:</t>
   </si>
   <si>
-    <t>• 3</t>
-  </si>
-  <si>
-    <t>• 4</t>
-  </si>
-  <si>
-    <t>• 5</t>
-  </si>
-  <si>
     <t>Tỉ số truyền của hộp số của động cơ M517 khi tiến là:</t>
   </si>
   <si>
-    <t>• 0,187</t>
-  </si>
-  <si>
-    <t>• 0,178</t>
-  </si>
-  <si>
-    <t>• 0,515</t>
-  </si>
-  <si>
-    <t>• 0,541</t>
-  </si>
-  <si>
     <t>Áp lực đóng mở ly hợp của động cơ M503 A:</t>
   </si>
   <si>
-    <t>• Tiến: 65 ÷ 78 kg/cm2; Lùi: 19 ÷ 24 kg/cm2</t>
-  </si>
-  <si>
-    <t>• Tiến: 65 ÷ 87 kg/cm2; Lùi: 19 ÷ 23 kg/cm2</t>
-  </si>
-  <si>
-    <t>• Tiến: 75 ÷ 92 kg/cm2; Lùi: 19 ÷ 24 kg/cm2</t>
-  </si>
-  <si>
-    <t>• Tiến: 75 ÷ 92 kg/cm2; Lùi: 19 ÷ 23 kg/cm2</t>
-  </si>
-  <si>
     <t>Tốc độ vòng quay lớn nhất của động cơ M520 là:</t>
   </si>
   <si>
@@ -322,12 +287,27 @@
   </si>
   <si>
     <t> 266ME</t>
+  </si>
+  <si>
+    <t>Ý 1 và 3</t>
+  </si>
+  <si>
+    <t>Tiến: 65 ÷ 78 kg/cm2; Lùi: 19 ÷ 24 kg/cm2</t>
+  </si>
+  <si>
+    <t>Tiến: 65 ÷ 87 kg/cm2; Lùi: 19 ÷ 23 kg/cm2</t>
+  </si>
+  <si>
+    <t>Tiến: 75 ÷ 92 kg/cm2; Lùi: 19 ÷ 24 kg/cm2</t>
+  </si>
+  <si>
+    <t>Tiến: 75 ÷ 92 kg/cm2; Lùi: 19 ÷ 23 kg/cm2</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
@@ -696,25 +676,25 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.35"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G28"/>
-  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:F25"/>
+  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="49.09765625" customWidth="1"/>
-    <col min="2" max="5" width="23.19921875" customWidth="1"/>
+    <col min="1" max="1" width="49.08203125" customWidth="1"/>
+    <col min="2" max="5" width="23.1640625" customWidth="1"/>
     <col min="6" max="6" width="11" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -733,11 +713,8 @@
       <c r="F1" s="4">
         <v>3</v>
       </c>
-      <c r="G1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
@@ -756,11 +733,8 @@
       <c r="F2" s="4">
         <v>1</v>
       </c>
-      <c r="G2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -774,16 +748,13 @@
         <v>9</v>
       </c>
       <c r="E3" t="s">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="F3" s="4">
         <v>4</v>
       </c>
-      <c r="G3">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="93.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:6" ht="90" x14ac:dyDescent="0.35">
       <c r="A4" s="8" t="s">
         <v>10</v>
       </c>
@@ -802,11 +773,8 @@
       <c r="F4" s="4">
         <v>4</v>
       </c>
-      <c r="G4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="20.25" x14ac:dyDescent="0.35">
+    </row>
+    <row r="5" spans="1:6" ht="20.399999999999999" x14ac:dyDescent="0.45">
       <c r="A5" s="5" t="s">
         <v>15</v>
       </c>
@@ -825,108 +793,93 @@
       <c r="F5" s="4">
         <v>2</v>
       </c>
-      <c r="G5">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="101.25" x14ac:dyDescent="0.3">
+    </row>
+    <row r="6" spans="1:6" ht="102" x14ac:dyDescent="0.35">
       <c r="A6" s="7" t="s">
         <v>16</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>58</v>
+        <v>46</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>59</v>
+        <v>47</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>17</v>
+        <v>87</v>
       </c>
       <c r="F6" s="4">
         <v>2</v>
       </c>
-      <c r="G6">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="20.25" x14ac:dyDescent="0.3">
+    </row>
+    <row r="7" spans="1:6" ht="20.399999999999999" x14ac:dyDescent="0.35">
       <c r="A7" s="7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="D7" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="E7" s="9" t="s">
-        <v>21</v>
+        <v>48</v>
+      </c>
+      <c r="C7" s="9">
+        <v>3</v>
+      </c>
+      <c r="D7" s="9">
+        <v>4</v>
+      </c>
+      <c r="E7" s="9">
+        <v>5</v>
       </c>
       <c r="F7" s="4">
         <v>2</v>
       </c>
-      <c r="G7">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="40.5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="8" spans="1:6" ht="40.799999999999997" x14ac:dyDescent="0.35">
       <c r="A8" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="D8" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="E8" s="9" t="s">
-        <v>26</v>
+        <v>18</v>
+      </c>
+      <c r="B8" s="9">
+        <v>0.187</v>
+      </c>
+      <c r="C8" s="9">
+        <v>0.17799999999999999</v>
+      </c>
+      <c r="D8" s="9">
+        <v>0.51500000000000001</v>
+      </c>
+      <c r="E8" s="9">
+        <v>0.54100000000000004</v>
       </c>
       <c r="F8" s="4">
         <v>3</v>
       </c>
-      <c r="G8">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="40.5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="9" spans="1:6" ht="40.799999999999997" x14ac:dyDescent="0.35">
       <c r="A9" s="7" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>28</v>
+        <v>88</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>29</v>
+        <v>89</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>31</v>
+        <v>91</v>
       </c>
       <c r="F9" s="4">
         <v>1</v>
       </c>
-      <c r="G9">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="10" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="7" t="s">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>82</v>
+        <v>70</v>
       </c>
       <c r="C10" s="6">
         <v>1950</v>
@@ -940,128 +893,110 @@
       <c r="F10" s="4">
         <v>4</v>
       </c>
-      <c r="G10">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="20.25" x14ac:dyDescent="0.3">
+    </row>
+    <row r="11" spans="1:6" ht="20.399999999999999" x14ac:dyDescent="0.35">
       <c r="A11" s="7" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>83</v>
+        <v>71</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>84</v>
+        <v>72</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>85</v>
+        <v>73</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
       <c r="F11" s="4">
         <v>1</v>
       </c>
-      <c r="G11">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="40.5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="12" spans="1:6" ht="40.799999999999997" x14ac:dyDescent="0.35">
       <c r="A12" s="7" t="s">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="F12" s="4">
         <v>3</v>
       </c>
-      <c r="G12">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="20.25" x14ac:dyDescent="0.3">
+    </row>
+    <row r="13" spans="1:6" ht="20.399999999999999" x14ac:dyDescent="0.35">
       <c r="A13" s="7" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>77</v>
+        <v>65</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>79</v>
+        <v>67</v>
       </c>
       <c r="F13" s="4">
         <v>2</v>
       </c>
-      <c r="G13">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="40.5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="14" spans="1:6" ht="40.799999999999997" x14ac:dyDescent="0.35">
       <c r="A14" s="7" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="F14" s="4">
         <v>4</v>
       </c>
-      <c r="G14">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="40.5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="15" spans="1:6" ht="40.799999999999997" x14ac:dyDescent="0.35">
       <c r="A15" s="7" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="F15" s="4">
         <v>4</v>
       </c>
-      <c r="G15">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="20.25" x14ac:dyDescent="0.3">
+    </row>
+    <row r="16" spans="1:6" ht="20.399999999999999" x14ac:dyDescent="0.35">
       <c r="A16" s="7" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="B16" s="6">
         <v>109</v>
@@ -1078,151 +1013,130 @@
       <c r="F16" s="4">
         <v>2</v>
       </c>
-      <c r="G16">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="60.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="17" spans="1:6" ht="61.2" x14ac:dyDescent="0.35">
       <c r="A17" s="7" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>90</v>
+        <v>78</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="F17" s="4">
         <v>3</v>
       </c>
-      <c r="G17">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="81" x14ac:dyDescent="0.3">
+    </row>
+    <row r="18" spans="1:6" ht="81.599999999999994" x14ac:dyDescent="0.35">
       <c r="A18" s="7" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>95</v>
+        <v>83</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>94</v>
+        <v>82</v>
       </c>
       <c r="F18" s="4">
         <v>1</v>
       </c>
-      <c r="G18">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" ht="40.5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="19" spans="1:6" ht="40.799999999999997" x14ac:dyDescent="0.35">
       <c r="A19" s="7" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>61</v>
+        <v>49</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>70</v>
+        <v>58</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>71</v>
+        <v>59</v>
       </c>
       <c r="F19" s="4">
         <v>3</v>
       </c>
-      <c r="G19">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" ht="40.5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="20" spans="1:6" ht="40.799999999999997" x14ac:dyDescent="0.35">
       <c r="A20" s="7" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>62</v>
+        <v>50</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>69</v>
+        <v>57</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>68</v>
+        <v>56</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="F20" s="4">
         <v>1</v>
       </c>
-      <c r="G20">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" ht="20.25" x14ac:dyDescent="0.3">
+    </row>
+    <row r="21" spans="1:6" ht="20.399999999999999" x14ac:dyDescent="0.35">
       <c r="A21" s="7" t="s">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>63</v>
+        <v>51</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>64</v>
+        <v>52</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>65</v>
+        <v>53</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>66</v>
+        <v>54</v>
       </c>
       <c r="F21" s="4">
         <v>4</v>
       </c>
-      <c r="G21">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" ht="40.5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="22" spans="1:6" ht="40.799999999999997" x14ac:dyDescent="0.35">
       <c r="A22" s="7" t="s">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>73</v>
+        <v>61</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="F22" s="4">
         <v>2</v>
       </c>
-      <c r="G22">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" ht="20.25" x14ac:dyDescent="0.3">
+    </row>
+    <row r="23" spans="1:6" ht="20.399999999999999" x14ac:dyDescent="0.35">
       <c r="A23" s="7" t="s">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="B23" s="6">
         <v>40</v>
@@ -1239,13 +1153,10 @@
       <c r="F23" s="4">
         <v>2</v>
       </c>
-      <c r="G23">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" ht="20.25" x14ac:dyDescent="0.3">
+    </row>
+    <row r="24" spans="1:6" ht="20.399999999999999" x14ac:dyDescent="0.35">
       <c r="A24" s="7" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="B24">
         <v>1</v>
@@ -1262,46 +1173,25 @@
       <c r="F24" s="4">
         <v>3</v>
       </c>
-      <c r="G24">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" ht="101.25" x14ac:dyDescent="0.3">
+    </row>
+    <row r="25" spans="1:6" ht="102" x14ac:dyDescent="0.35">
       <c r="A25" s="7" t="s">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="F25" s="4">
         <v>3</v>
-      </c>
-      <c r="G25">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="G26">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="G27">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="G28">
-        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>